<commit_message>
comex, + cdg y update proyecto
</commit_message>
<xml_diff>
--- a/2026/Proyecto_Final/drive_proyecto_final/Técnico/BOM Productos.xlsx
+++ b/2026/Proyecto_Final/drive_proyecto_final/Técnico/BOM Productos.xlsx
@@ -13,10 +13,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={bbfc8462-757c-471e-930f-9b1c48445796}</author>
+    <author>tc={180e2472-7d68-4565-af40-1daa5c32d32e}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{bbfc8462-757c-471e-930f-9b1c48445796}" ref="D96">
+    <comment authorId="0" xr:uid="{180e2472-7d68-4565-af40-1daa5c32d32e}" ref="D96">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1613,7 +1613,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Mateo AlbarracÍn" id="{f68bb5ed-703d-4b51-90c8-78e65b7d0540}" providerId="google-sheets"/>
+  <x18tc:person displayName="Mateo AlbarracÍn" id="{ef50f02f-2d6f-4d06-a5d7-95fde7328dac}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1813,7 +1813,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="D96" dT="2026-06-23T22:31:01.00" personId="{f68bb5ed-703d-4b51-90c8-78e65b7d0540}" id="{bbfc8462-757c-471e-930f-9b1c48445796}" done="0">
+  <x18tc:threadedComment ref="D96" dT="2026-06-23T22:31:01.00" personId="{ef50f02f-2d6f-4d06-a5d7-95fde7328dac}" id="{180e2472-7d68-4565-af40-1daa5c32d32e}" done="0">
     <x18tc:text xml:space="preserve">Es bastante bajo. Analizar agua</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>

</xml_diff>